<commit_message>
Apply confirmed accountant decisions to UVG invoice imports
Add 48 proposed invoices on 27 roots, preserve whole excluded chains, and retain source replies and XML evidence. Include independent final verification, pre-update baselines, and current cross-machine handoff instructions.
</commit_message>
<xml_diff>
--- a/outputs/NGOAI_LE_F0_2024_T6_2025.xlsx
+++ b/outputs/NGOAI_LE_F0_2024_T6_2025.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ngoai le" sheetId="1" r:id="Rcd83779b2eb44384"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huong dan" sheetId="2" r:id="R484565a2ac534637"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chi tiet nguon" sheetId="3" r:id="R64dced52e6b84fef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ngoai le" sheetId="1" r:id="R88ce1ca00f254e30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huong dan" sheetId="2" r:id="R349f3a73c38a49e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chi tiet nguon" sheetId="3" r:id="R8825031f5f7e4cd2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -80,7 +80,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="22">
+  <x:cellXfs count="26">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -141,6 +141,18 @@
     <x:xf numFmtId="200" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -149,8 +161,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="NgoaiLeChuoi" displayName="NgoaiLeChuoi" ref="A2:X240" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A2:X240"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="NgoaiLeChuoi" displayName="NgoaiLeChuoi" ref="A2:X246" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A2:X246"/>
   <x:tableColumns count="24">
     <x:tableColumn id="1" name="Tên người mua"/>
     <x:tableColumn id="2" name="MST/CCCD chủ hộ nguyên bản"/>
@@ -182,8 +194,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="NguonNgoaiLe" displayName="NguonNgoaiLe" ref="A1:M327" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:M327"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NguonNgoaiLe" displayName="NguonNgoaiLe" ref="A1:M339" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:M339"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Ký hiệu gốc"/>
     <x:tableColumn id="2" name="Số gốc"/>
@@ -13044,6 +13056,350 @@
       </x:c>
       <x:c r="X240" s="9" t="str"/>
     </x:row>
+    <x:row r="241" ht="110" customHeight="1">
+      <x:c r="A241" s="9" t="str">
+        <x:v>Khách lẻ không lấy hóa đơn</x:v>
+      </x:c>
+      <x:c r="B241" s="9" t="str"/>
+      <x:c r="C241" s="9" t="str">
+        <x:v>1C24TUV</x:v>
+      </x:c>
+      <x:c r="D241" s="24" t="str">
+        <x:v>00000003</x:v>
+      </x:c>
+      <x:c r="E241" s="23" t="d">
+        <x:v>2024-01-10T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F241" s="25" t="n">
+        <x:v>11334130</x:v>
+      </x:c>
+      <x:c r="G241" s="25" t="n">
+        <x:v>906730</x:v>
+      </x:c>
+      <x:c r="H241" s="25" t="n">
+        <x:v>12240860</x:v>
+      </x:c>
+      <x:c r="I241" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="J241" s="24" t="str">
+        <x:v>00000508</x:v>
+      </x:c>
+      <x:c r="K241" s="23" t="d">
+        <x:v>2025-04-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="L241" s="25" t="n">
+        <x:v>-356085</x:v>
+      </x:c>
+      <x:c r="M241" s="25" t="n">
+        <x:v>-28487</x:v>
+      </x:c>
+      <x:c r="N241" s="25" t="n">
+        <x:v>-384572</x:v>
+      </x:c>
+      <x:c r="O241" s="9"/>
+      <x:c r="P241" s="24"/>
+      <x:c r="Q241" s="23"/>
+      <x:c r="R241" s="25"/>
+      <x:c r="S241" s="25"/>
+      <x:c r="T241" s="25"/>
+      <x:c r="U241" s="25" t="n">
+        <x:v>10978045</x:v>
+      </x:c>
+      <x:c r="V241" s="25" t="n">
+        <x:v>878243</x:v>
+      </x:c>
+      <x:c r="W241" s="25" t="n">
+        <x:v>11856288</x:v>
+      </x:c>
+      <x:c r="X241" s="9" t="str">
+        <x:v>Giữ nguyên toàn bộ chuỗi theo xác nhận điểm 6; không lập điều chỉnh mới.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="242" ht="110" customHeight="1">
+      <x:c r="A242" s="9" t="str">
+        <x:v>Khách lẻ không lấy hoá đơn</x:v>
+      </x:c>
+      <x:c r="B242" s="9" t="str"/>
+      <x:c r="C242" s="9" t="str">
+        <x:v>1C24TUV</x:v>
+      </x:c>
+      <x:c r="D242" s="24" t="str">
+        <x:v>00000498</x:v>
+      </x:c>
+      <x:c r="E242" s="23" t="d">
+        <x:v>2024-09-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F242" s="25" t="n">
+        <x:v>197727562</x:v>
+      </x:c>
+      <x:c r="G242" s="25" t="n">
+        <x:v>15818205</x:v>
+      </x:c>
+      <x:c r="H242" s="25" t="n">
+        <x:v>213545767</x:v>
+      </x:c>
+      <x:c r="I242" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="J242" s="24" t="str">
+        <x:v>00002140</x:v>
+      </x:c>
+      <x:c r="K242" s="23" t="d">
+        <x:v>2025-05-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="L242" s="25" t="n">
+        <x:v>17830586</x:v>
+      </x:c>
+      <x:c r="M242" s="25" t="n">
+        <x:v>1426447</x:v>
+      </x:c>
+      <x:c r="N242" s="25" t="n">
+        <x:v>19257033</x:v>
+      </x:c>
+      <x:c r="O242" s="9"/>
+      <x:c r="P242" s="24"/>
+      <x:c r="Q242" s="23"/>
+      <x:c r="R242" s="25"/>
+      <x:c r="S242" s="25"/>
+      <x:c r="T242" s="25"/>
+      <x:c r="U242" s="25" t="n">
+        <x:v>215558148</x:v>
+      </x:c>
+      <x:c r="V242" s="25" t="n">
+        <x:v>17244652</x:v>
+      </x:c>
+      <x:c r="W242" s="25" t="n">
+        <x:v>232802800</x:v>
+      </x:c>
+      <x:c r="X242" s="9" t="str">
+        <x:v>Giữ nguyên toàn bộ chuỗi theo xác nhận điểm 6; không lập điều chỉnh mới.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="243" ht="110" customHeight="1">
+      <x:c r="A243" s="9" t="str">
+        <x:v>Khách lẻ không lấy hóa đơn</x:v>
+      </x:c>
+      <x:c r="B243" s="9" t="str"/>
+      <x:c r="C243" s="9" t="str">
+        <x:v>1C24TUV</x:v>
+      </x:c>
+      <x:c r="D243" s="24" t="str">
+        <x:v>00000574</x:v>
+      </x:c>
+      <x:c r="E243" s="23" t="d">
+        <x:v>2024-11-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F243" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G243" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H243" s="25"/>
+      <x:c r="I243" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="J243" s="24" t="str">
+        <x:v>00002189</x:v>
+      </x:c>
+      <x:c r="K243" s="23" t="d">
+        <x:v>2025-05-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="L243" s="25" t="n">
+        <x:v>1702778</x:v>
+      </x:c>
+      <x:c r="M243" s="25" t="n">
+        <x:v>136222</x:v>
+      </x:c>
+      <x:c r="N243" s="25" t="n">
+        <x:v>1839000</x:v>
+      </x:c>
+      <x:c r="O243" s="9"/>
+      <x:c r="P243" s="24"/>
+      <x:c r="Q243" s="23"/>
+      <x:c r="R243" s="25"/>
+      <x:c r="S243" s="25"/>
+      <x:c r="T243" s="25"/>
+      <x:c r="U243" s="25" t="n">
+        <x:v>1702778</x:v>
+      </x:c>
+      <x:c r="V243" s="25" t="n">
+        <x:v>136222</x:v>
+      </x:c>
+      <x:c r="W243" s="25"/>
+      <x:c r="X243" s="9" t="str">
+        <x:v>Giữ nguyên toàn bộ chuỗi theo xác nhận điểm 6; không lập điều chỉnh mới.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="244" ht="110" customHeight="1">
+      <x:c r="A244" s="9" t="str">
+        <x:v>KHÁCH HÀNG LẺ SP - KHÔNG LẤY HÓA ĐƠN</x:v>
+      </x:c>
+      <x:c r="B244" s="9" t="str"/>
+      <x:c r="C244" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="D244" s="24" t="str">
+        <x:v>00001348</x:v>
+      </x:c>
+      <x:c r="E244" s="23" t="d">
+        <x:v>2025-05-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F244" s="25" t="n">
+        <x:v>675000</x:v>
+      </x:c>
+      <x:c r="G244" s="25" t="n">
+        <x:v>54000</x:v>
+      </x:c>
+      <x:c r="H244" s="25" t="n">
+        <x:v>729000</x:v>
+      </x:c>
+      <x:c r="I244" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="J244" s="24" t="str">
+        <x:v>00006108</x:v>
+      </x:c>
+      <x:c r="K244" s="23" t="d">
+        <x:v>2025-06-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="L244" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M244" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N244" s="25"/>
+      <x:c r="O244" s="9"/>
+      <x:c r="P244" s="24"/>
+      <x:c r="Q244" s="23"/>
+      <x:c r="R244" s="25"/>
+      <x:c r="S244" s="25"/>
+      <x:c r="T244" s="25"/>
+      <x:c r="U244" s="25" t="n">
+        <x:v>675000</x:v>
+      </x:c>
+      <x:c r="V244" s="25" t="n">
+        <x:v>54000</x:v>
+      </x:c>
+      <x:c r="W244" s="25"/>
+      <x:c r="X244" s="9" t="str">
+        <x:v>Giữ nguyên toàn bộ chuỗi theo xác nhận điểm 6; không lập điều chỉnh mới.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="245" ht="110" customHeight="1">
+      <x:c r="A245" s="9" t="str">
+        <x:v>KHÁCH HÀNG LẺ SP - KHÔNG LẤY HÓA ĐƠN</x:v>
+      </x:c>
+      <x:c r="B245" s="9" t="str"/>
+      <x:c r="C245" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="D245" s="24" t="str">
+        <x:v>00002377</x:v>
+      </x:c>
+      <x:c r="E245" s="23" t="d">
+        <x:v>2025-05-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F245" s="25" t="n">
+        <x:v>406481</x:v>
+      </x:c>
+      <x:c r="G245" s="25" t="n">
+        <x:v>32518</x:v>
+      </x:c>
+      <x:c r="H245" s="25" t="n">
+        <x:v>438999</x:v>
+      </x:c>
+      <x:c r="I245" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="J245" s="24" t="str">
+        <x:v>00004203</x:v>
+      </x:c>
+      <x:c r="K245" s="23" t="d">
+        <x:v>2025-06-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="L245" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M245" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N245" s="25"/>
+      <x:c r="O245" s="9"/>
+      <x:c r="P245" s="24"/>
+      <x:c r="Q245" s="23"/>
+      <x:c r="R245" s="25"/>
+      <x:c r="S245" s="25"/>
+      <x:c r="T245" s="25"/>
+      <x:c r="U245" s="25" t="n">
+        <x:v>406481</x:v>
+      </x:c>
+      <x:c r="V245" s="25" t="n">
+        <x:v>32518</x:v>
+      </x:c>
+      <x:c r="W245" s="25"/>
+      <x:c r="X245" s="9" t="str">
+        <x:v>Giữ nguyên toàn bộ chuỗi theo xác nhận điểm 6; không lập điều chỉnh mới.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="246" ht="110" customHeight="1">
+      <x:c r="A246" s="9" t="str">
+        <x:v>KHÁCH HÀNG LẺ SP - KHÔNG LẤY HÓA ĐƠN</x:v>
+      </x:c>
+      <x:c r="B246" s="9" t="str"/>
+      <x:c r="C246" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="D246" s="24" t="str">
+        <x:v>00002378</x:v>
+      </x:c>
+      <x:c r="E246" s="23" t="d">
+        <x:v>2025-05-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F246" s="25" t="n">
+        <x:v>406481</x:v>
+      </x:c>
+      <x:c r="G246" s="25" t="n">
+        <x:v>32518</x:v>
+      </x:c>
+      <x:c r="H246" s="25" t="n">
+        <x:v>438999</x:v>
+      </x:c>
+      <x:c r="I246" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="J246" s="24" t="str">
+        <x:v>00004204</x:v>
+      </x:c>
+      <x:c r="K246" s="23" t="d">
+        <x:v>2025-06-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="L246" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M246" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N246" s="25"/>
+      <x:c r="O246" s="9"/>
+      <x:c r="P246" s="24"/>
+      <x:c r="Q246" s="23"/>
+      <x:c r="R246" s="25"/>
+      <x:c r="S246" s="25"/>
+      <x:c r="T246" s="25"/>
+      <x:c r="U246" s="25" t="n">
+        <x:v>406481</x:v>
+      </x:c>
+      <x:c r="V246" s="25" t="n">
+        <x:v>32518</x:v>
+      </x:c>
+      <x:c r="W246" s="25"/>
+      <x:c r="X246" s="9" t="str">
+        <x:v>Giữ nguyên toàn bộ chuỗi theo xác nhận điểm 6; không lập điều chỉnh mới.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:B1"/>
@@ -13054,7 +13410,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f65f085789442fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fd8fad4d83d4a78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13073,22 +13429,22 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="9" t="str">
-        <x:v>F0 từ 01/01/2024 đến 30/06/2025; hóa đơn liên quan đến 31/12/2025.</x:v>
+        <x:v>F0 từ 01/01/2024 đến 30/06/2025. Quy tắc giữ nguyên được rà thêm theo các liên kết và thay đổi người mua trong dữ liệu xuất lại đến 09/10/2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="9" t="str">
-        <x:v>238 F0, 326 hóa đơn riêng biệt; 2 chuỗi có ghi chú cần kiểm tra.</x:v>
+        <x:v>244 chuỗi giữ nguyên / 338 hóa đơn liên quan: gồm 238 ngoại lệ trước và 6 cặp vừa được chốt giữ nguyên toàn bộ.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
       <x:c r="A4" s="9" t="str">
-        <x:v>F0 năm 2024: 118; F0 tháng 1–6/2025: 120.</x:v>
+        <x:v>F0 năm 2024: 121; F0 tháng 1–6/2025: 123.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="9" t="str">
-        <x:v>Ngoại lệ nhận diện bằng tên công ty/doanh nghiệp hoặc định danh dạng MST trong nguồn; chưa xác thực MST.</x:v>
+        <x:v>Giữ nguyên toàn chuỗi theo tên công ty/hộ kinh doanh, định danh thuộc quy tắc ngoại lệ trước, các lần điều chỉnh đổi người mua và 6 cặp được chỉ định giữ nguyên.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
@@ -13116,14 +13472,14 @@
         <x:v>18 file nguồn có SHA-256 trong SOURCE_MANIFEST.json; 8 liên kết lịch sử bổ sung từ Git có vị trí nguồn.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="34" customHeight="1">
+    <x:row r="11" ht="65" customHeight="1">
       <x:c r="A11" s="9" t="str">
-        <x:v>0 F0 ngoài ngoại lệ có nhãn đã xử lý nhưng chưa có liên kết đến 31/12/2025; không tự đưa vào nhóm đã điều chỉnh.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="34" customHeight="1">
+        <x:v>Theo chốt điểm6: giữ mọi hóa đơn trong chuỗi nếu bất kỳ hóa đơn nào xuất cho công ty/hộ kinh doanh hoặc đã đổi người mua thành công ty/hộ kinh doanh. Giữ thêm6cặp được chỉ định, gồm3/508.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="65" customHeight="1">
       <x:c r="A12" s="9" t="str">
-        <x:v>Đơn vị: đồng. Đây là bảng rà soát; chưa chốt nghiệp vụ phát hành, chưa tạo import, ký hoặc phát hành hóa đơn.</x:v>
+        <x:v>6 chuỗi mới được thêm ở cuối Ngoai le và Chi tiet nguon; bảng đã điều chỉnh vẫn lưu nguồn lịch sử nhưng đã xóa phương án phát sinh cho các chuỗi này. Không có hóa đơn thuộc diện giữ nguyên trong hai bảng import.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -26555,10 +26911,470 @@
         <x:v>data/Du lieu Meinvoice/Bang_ke_hoa_don_da_su_dung_2024_2025/Bang_ke_hoa_don_da_su_dung_1791380301707_3.xlsx | dòng 275</x:v>
       </x:c>
     </x:row>
+    <x:row r="328" ht="90" customHeight="1">
+      <x:c r="A328" s="9" t="str">
+        <x:v>1C24TUV</x:v>
+      </x:c>
+      <x:c r="B328" s="9" t="str">
+        <x:v>00000003</x:v>
+      </x:c>
+      <x:c r="C328" s="9" t="str">
+        <x:v>1C24TUV</x:v>
+      </x:c>
+      <x:c r="D328" s="9" t="str">
+        <x:v>00000003</x:v>
+      </x:c>
+      <x:c r="E328" s="23" t="d">
+        <x:v>2024-01-10T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F328" s="9" t="str">
+        <x:v>Khách lẻ không lấy hóa đơn</x:v>
+      </x:c>
+      <x:c r="G328" s="9" t="str"/>
+      <x:c r="H328" s="9" t="str">
+        <x:v>Hóa đơn gốc</x:v>
+      </x:c>
+      <x:c r="I328" s="9" t="str">
+        <x:v>Hóa đơn đã bị điều chỉnh</x:v>
+      </x:c>
+      <x:c r="J328" s="25" t="n">
+        <x:v>11334130</x:v>
+      </x:c>
+      <x:c r="K328" s="25" t="n">
+        <x:v>906730</x:v>
+      </x:c>
+      <x:c r="L328" s="25" t="n">
+        <x:v>12240860</x:v>
+      </x:c>
+      <x:c r="M328" s="9" t="str">
+        <x:v>data/Du lieu Meinvoice/Xuat_lai_2026-10-09/Bang_ke_hoa_don_da_su_dung_1791532882546.xlsx | dòng 8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="329" ht="90" customHeight="1">
+      <x:c r="A329" s="9" t="str">
+        <x:v>1C24TUV</x:v>
+      </x:c>
+      <x:c r="B329" s="9" t="str">
+        <x:v>00000003</x:v>
+      </x:c>
+      <x:c r="C329" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="D329" s="9" t="str">
+        <x:v>00000508</x:v>
+      </x:c>
+      <x:c r="E329" s="23" t="d">
+        <x:v>2025-04-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F329" s="9" t="str">
+        <x:v>Khách lẻ không lấy hóa đơn</x:v>
+      </x:c>
+      <x:c r="G329" s="9" t="str"/>
+      <x:c r="H329" s="9" t="str">
+        <x:v>Điều chỉnh; giữ nguyên cả chuỗi theo xác nhận</x:v>
+      </x:c>
+      <x:c r="I329" s="9" t="str">
+        <x:v>Hoá đơn điều chỉnh</x:v>
+      </x:c>
+      <x:c r="J329" s="25" t="n">
+        <x:v>-356085</x:v>
+      </x:c>
+      <x:c r="K329" s="25" t="n">
+        <x:v>-28487</x:v>
+      </x:c>
+      <x:c r="L329" s="25" t="n">
+        <x:v>-384572</x:v>
+      </x:c>
+      <x:c r="M329" s="9" t="str">
+        <x:v>data/Du lieu Meinvoice/Xuat_lai_2026-10-09/Bang_ke_hoa_don_da_su_dung_1791532908545.zip / Bang_ke_hoa_don_da_su_dung_1791532908545_1.xlsx | dòng 513</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="330" ht="90" customHeight="1">
+      <x:c r="A330" s="9" t="str">
+        <x:v>1C24TUV</x:v>
+      </x:c>
+      <x:c r="B330" s="9" t="str">
+        <x:v>00000498</x:v>
+      </x:c>
+      <x:c r="C330" s="9" t="str">
+        <x:v>1C24TUV</x:v>
+      </x:c>
+      <x:c r="D330" s="9" t="str">
+        <x:v>00000498</x:v>
+      </x:c>
+      <x:c r="E330" s="23" t="d">
+        <x:v>2024-09-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F330" s="9" t="str">
+        <x:v>Khách lẻ không lấy hoá đơn</x:v>
+      </x:c>
+      <x:c r="G330" s="9" t="str"/>
+      <x:c r="H330" s="9" t="str">
+        <x:v>Hóa đơn gốc</x:v>
+      </x:c>
+      <x:c r="I330" s="9" t="str">
+        <x:v>Hóa đơn đã bị điều chỉnh</x:v>
+      </x:c>
+      <x:c r="J330" s="25" t="n">
+        <x:v>197727562</x:v>
+      </x:c>
+      <x:c r="K330" s="25" t="n">
+        <x:v>15818205</x:v>
+      </x:c>
+      <x:c r="L330" s="25" t="n">
+        <x:v>213545767</x:v>
+      </x:c>
+      <x:c r="M330" s="9" t="str">
+        <x:v>data/Du lieu Meinvoice/Xuat_lai_2026-10-09/Bang_ke_hoa_don_da_su_dung_1791532882546.xlsx | dòng 503</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="331" ht="90" customHeight="1">
+      <x:c r="A331" s="9" t="str">
+        <x:v>1C24TUV</x:v>
+      </x:c>
+      <x:c r="B331" s="9" t="str">
+        <x:v>00000498</x:v>
+      </x:c>
+      <x:c r="C331" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="D331" s="9" t="str">
+        <x:v>00002140</x:v>
+      </x:c>
+      <x:c r="E331" s="23" t="d">
+        <x:v>2025-05-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F331" s="9" t="str">
+        <x:v>Khách lẻ không lấy hoá đơn</x:v>
+      </x:c>
+      <x:c r="G331" s="9" t="str"/>
+      <x:c r="H331" s="9" t="str">
+        <x:v>Điều chỉnh; giữ nguyên cả chuỗi theo xác nhận</x:v>
+      </x:c>
+      <x:c r="I331" s="9" t="str">
+        <x:v>Hoá đơn điều chỉnh</x:v>
+      </x:c>
+      <x:c r="J331" s="25" t="n">
+        <x:v>17830586</x:v>
+      </x:c>
+      <x:c r="K331" s="25" t="n">
+        <x:v>1426447</x:v>
+      </x:c>
+      <x:c r="L331" s="25" t="n">
+        <x:v>19257033</x:v>
+      </x:c>
+      <x:c r="M331" s="9" t="str">
+        <x:v>data/Du lieu Meinvoice/Xuat_lai_2026-10-09/Bang_ke_hoa_don_da_su_dung_1791532908545.zip / Bang_ke_hoa_don_da_su_dung_1791532908545_1.xlsx | dòng 2145</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="332" ht="90" customHeight="1">
+      <x:c r="A332" s="9" t="str">
+        <x:v>1C24TUV</x:v>
+      </x:c>
+      <x:c r="B332" s="9" t="str">
+        <x:v>00000574</x:v>
+      </x:c>
+      <x:c r="C332" s="9" t="str">
+        <x:v>1C24TUV</x:v>
+      </x:c>
+      <x:c r="D332" s="9" t="str">
+        <x:v>00000574</x:v>
+      </x:c>
+      <x:c r="E332" s="23" t="d">
+        <x:v>2024-11-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F332" s="9" t="str">
+        <x:v>Khách lẻ không lấy hóa đơn</x:v>
+      </x:c>
+      <x:c r="G332" s="9" t="str"/>
+      <x:c r="H332" s="9" t="str">
+        <x:v>Hóa đơn gốc</x:v>
+      </x:c>
+      <x:c r="I332" s="9" t="str">
+        <x:v>Hóa đơn đã bị điều chỉnh</x:v>
+      </x:c>
+      <x:c r="J332" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K332" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L332" s="25"/>
+      <x:c r="M332" s="9" t="str">
+        <x:v>data/Du lieu Meinvoice/Xuat_lai_2026-10-09/Bang_ke_hoa_don_da_su_dung_1791532882546.xlsx | dòng 579</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="333" ht="90" customHeight="1">
+      <x:c r="A333" s="9" t="str">
+        <x:v>1C24TUV</x:v>
+      </x:c>
+      <x:c r="B333" s="9" t="str">
+        <x:v>00000574</x:v>
+      </x:c>
+      <x:c r="C333" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="D333" s="9" t="str">
+        <x:v>00002189</x:v>
+      </x:c>
+      <x:c r="E333" s="23" t="d">
+        <x:v>2025-05-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F333" s="9" t="str">
+        <x:v>Khách lẻ không lấy hóa đơn</x:v>
+      </x:c>
+      <x:c r="G333" s="9" t="str"/>
+      <x:c r="H333" s="9" t="str">
+        <x:v>Điều chỉnh; giữ nguyên cả chuỗi theo xác nhận</x:v>
+      </x:c>
+      <x:c r="I333" s="9" t="str">
+        <x:v>Hoá đơn điều chỉnh</x:v>
+      </x:c>
+      <x:c r="J333" s="25" t="n">
+        <x:v>1702778</x:v>
+      </x:c>
+      <x:c r="K333" s="25" t="n">
+        <x:v>136222</x:v>
+      </x:c>
+      <x:c r="L333" s="25" t="n">
+        <x:v>1839000</x:v>
+      </x:c>
+      <x:c r="M333" s="9" t="str">
+        <x:v>data/Du lieu Meinvoice/Xuat_lai_2026-10-09/Bang_ke_hoa_don_da_su_dung_1791532908545.zip / Bang_ke_hoa_don_da_su_dung_1791532908545_1.xlsx | dòng 2194</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="334" ht="90" customHeight="1">
+      <x:c r="A334" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="B334" s="9" t="str">
+        <x:v>00001348</x:v>
+      </x:c>
+      <x:c r="C334" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="D334" s="9" t="str">
+        <x:v>00001348</x:v>
+      </x:c>
+      <x:c r="E334" s="23" t="d">
+        <x:v>2025-05-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F334" s="9" t="str">
+        <x:v>KHÁCH HÀNG LẺ SP - KHÔNG LẤY HÓA ĐƠN</x:v>
+      </x:c>
+      <x:c r="G334" s="9" t="str"/>
+      <x:c r="H334" s="9" t="str">
+        <x:v>Hóa đơn gốc</x:v>
+      </x:c>
+      <x:c r="I334" s="9" t="str">
+        <x:v>Hóa đơn đã bị điều chỉnh</x:v>
+      </x:c>
+      <x:c r="J334" s="25" t="n">
+        <x:v>675000</x:v>
+      </x:c>
+      <x:c r="K334" s="25" t="n">
+        <x:v>54000</x:v>
+      </x:c>
+      <x:c r="L334" s="25" t="n">
+        <x:v>729000</x:v>
+      </x:c>
+      <x:c r="M334" s="9" t="str">
+        <x:v>data/Du lieu Meinvoice/Xuat_lai_2026-10-09/Bang_ke_hoa_don_da_su_dung_1791532908545.zip / Bang_ke_hoa_don_da_su_dung_1791532908545_1.xlsx | dòng 1353</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="335" ht="90" customHeight="1">
+      <x:c r="A335" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="B335" s="9" t="str">
+        <x:v>00001348</x:v>
+      </x:c>
+      <x:c r="C335" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="D335" s="9" t="str">
+        <x:v>00006108</x:v>
+      </x:c>
+      <x:c r="E335" s="23" t="d">
+        <x:v>2025-06-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F335" s="9" t="str">
+        <x:v>KHÁCH HÀNG LẺ SP - KHÔNG LẤY HÓA ĐƠN</x:v>
+      </x:c>
+      <x:c r="G335" s="9" t="str"/>
+      <x:c r="H335" s="9" t="str">
+        <x:v>Điều chỉnh; giữ nguyên cả chuỗi theo xác nhận</x:v>
+      </x:c>
+      <x:c r="I335" s="9" t="str">
+        <x:v>Hoá đơn điều chỉnh</x:v>
+      </x:c>
+      <x:c r="J335" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K335" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L335" s="25"/>
+      <x:c r="M335" s="9" t="str">
+        <x:v>data/Du lieu Meinvoice/Xuat_lai_2026-10-09/Bang_ke_hoa_don_da_su_dung_1791532908545.zip / Bang_ke_hoa_don_da_su_dung_1791532908545_2.xlsx | dòng 1200</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="336" ht="90" customHeight="1">
+      <x:c r="A336" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="B336" s="9" t="str">
+        <x:v>00002377</x:v>
+      </x:c>
+      <x:c r="C336" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="D336" s="9" t="str">
+        <x:v>00002377</x:v>
+      </x:c>
+      <x:c r="E336" s="23" t="d">
+        <x:v>2025-05-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F336" s="9" t="str">
+        <x:v>KHÁCH HÀNG LẺ SP - KHÔNG LẤY HÓA ĐƠN</x:v>
+      </x:c>
+      <x:c r="G336" s="9" t="str"/>
+      <x:c r="H336" s="9" t="str">
+        <x:v>Hóa đơn gốc</x:v>
+      </x:c>
+      <x:c r="I336" s="9" t="str">
+        <x:v>Hóa đơn đã bị điều chỉnh</x:v>
+      </x:c>
+      <x:c r="J336" s="25" t="n">
+        <x:v>406481</x:v>
+      </x:c>
+      <x:c r="K336" s="25" t="n">
+        <x:v>32518</x:v>
+      </x:c>
+      <x:c r="L336" s="25" t="n">
+        <x:v>438999</x:v>
+      </x:c>
+      <x:c r="M336" s="9" t="str">
+        <x:v>data/Du lieu Meinvoice/Xuat_lai_2026-10-09/Bang_ke_hoa_don_da_su_dung_1791532908545.zip / Bang_ke_hoa_don_da_su_dung_1791532908545_1.xlsx | dòng 2382</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="337" ht="90" customHeight="1">
+      <x:c r="A337" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="B337" s="9" t="str">
+        <x:v>00002377</x:v>
+      </x:c>
+      <x:c r="C337" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="D337" s="9" t="str">
+        <x:v>00004203</x:v>
+      </x:c>
+      <x:c r="E337" s="23" t="d">
+        <x:v>2025-06-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F337" s="9" t="str">
+        <x:v>KHÁCH HÀNG LẺ SP - KHÔNG LẤY HÓA ĐƠN</x:v>
+      </x:c>
+      <x:c r="G337" s="9" t="str"/>
+      <x:c r="H337" s="9" t="str">
+        <x:v>Điều chỉnh; giữ nguyên cả chuỗi theo xác nhận</x:v>
+      </x:c>
+      <x:c r="I337" s="9" t="str">
+        <x:v>Hoá đơn điều chỉnh</x:v>
+      </x:c>
+      <x:c r="J337" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K337" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L337" s="25"/>
+      <x:c r="M337" s="9" t="str">
+        <x:v>data/Du lieu Meinvoice/Xuat_lai_2026-10-09/Bang_ke_hoa_don_da_su_dung_1791532908545.zip / Bang_ke_hoa_don_da_su_dung_1791532908545_1.xlsx | dòng 4208</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="338" ht="90" customHeight="1">
+      <x:c r="A338" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="B338" s="9" t="str">
+        <x:v>00002378</x:v>
+      </x:c>
+      <x:c r="C338" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="D338" s="9" t="str">
+        <x:v>00002378</x:v>
+      </x:c>
+      <x:c r="E338" s="23" t="d">
+        <x:v>2025-05-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F338" s="9" t="str">
+        <x:v>KHÁCH HÀNG LẺ SP - KHÔNG LẤY HÓA ĐƠN</x:v>
+      </x:c>
+      <x:c r="G338" s="9" t="str"/>
+      <x:c r="H338" s="9" t="str">
+        <x:v>Hóa đơn gốc</x:v>
+      </x:c>
+      <x:c r="I338" s="9" t="str">
+        <x:v>Hóa đơn đã bị điều chỉnh</x:v>
+      </x:c>
+      <x:c r="J338" s="25" t="n">
+        <x:v>406481</x:v>
+      </x:c>
+      <x:c r="K338" s="25" t="n">
+        <x:v>32518</x:v>
+      </x:c>
+      <x:c r="L338" s="25" t="n">
+        <x:v>438999</x:v>
+      </x:c>
+      <x:c r="M338" s="9" t="str">
+        <x:v>data/Du lieu Meinvoice/Xuat_lai_2026-10-09/Bang_ke_hoa_don_da_su_dung_1791532908545.zip / Bang_ke_hoa_don_da_su_dung_1791532908545_1.xlsx | dòng 2383</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="339" ht="90" customHeight="1">
+      <x:c r="A339" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="B339" s="9" t="str">
+        <x:v>00002378</x:v>
+      </x:c>
+      <x:c r="C339" s="9" t="str">
+        <x:v>1C25TUV</x:v>
+      </x:c>
+      <x:c r="D339" s="9" t="str">
+        <x:v>00004204</x:v>
+      </x:c>
+      <x:c r="E339" s="23" t="d">
+        <x:v>2025-06-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F339" s="9" t="str">
+        <x:v>KHÁCH HÀNG LẺ SP - KHÔNG LẤY HÓA ĐƠN</x:v>
+      </x:c>
+      <x:c r="G339" s="9" t="str"/>
+      <x:c r="H339" s="9" t="str">
+        <x:v>Điều chỉnh; giữ nguyên cả chuỗi theo xác nhận</x:v>
+      </x:c>
+      <x:c r="I339" s="9" t="str">
+        <x:v>Hoá đơn điều chỉnh</x:v>
+      </x:c>
+      <x:c r="J339" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K339" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L339" s="25"/>
+      <x:c r="M339" s="9" t="str">
+        <x:v>data/Du lieu Meinvoice/Xuat_lai_2026-10-09/Bang_ke_hoa_don_da_su_dung_1791532908545.zip / Bang_ke_hoa_don_da_su_dung_1791532908545_1.xlsx | dòng 4209</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ffad4e251e5420d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d8af4576dbc4388"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>